<commit_message>
Integrate with main system
</commit_message>
<xml_diff>
--- a/template/WritOfSummons/Writ_of_Summons_Data_filled.xlsx
+++ b/template/WritOfSummons/Writ_of_Summons_Data_filled.xlsx
@@ -583,67 +583,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-08</t>
+          <t xml:space="preserve">2026-04-09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High Court</t>
+          <t xml:space="preserve">fgfgfgfgf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KL</t>
+          <t xml:space="preserve">fgfgfgfgfg</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">X-1</t>
+          <t xml:space="preserve">2365</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alice</t>
+          <t xml:space="preserve">sdfdsfsdf</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">900101-01-1111</t>
+          <t xml:space="preserve">030506090845</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dfdferr</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dfsetfe</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bob</t>
+          <t xml:space="preserve">dfseg</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">800101-01-2222</t>
+          <t xml:space="preserve">01020304056</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dgfgfg</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">fgfgfg</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5000</t>
+          <t xml:space="preserve">10205</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -653,67 +653,67 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dvsdvfhgfghbhfgjgfhn fgjhdfxgfhdgbdzfg thbgdfghn khmk hfdhbfdabgn ulkymaehf b rth fhn mhte r nmuhkythhgg, j.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-04-06</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">adfhggfsjfdh yghnmuy,dygjrts hytjnbrebtntrhrgehtr</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3.6</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">10000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">imsn</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Adnan Sharida</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">fgfgfgf fgfgfg fgfgfg fgfgf gfgfg</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0123659988</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">taimanaliff@gmail.com</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-04-14</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">dsvdd</t>
         </is>
       </c>
     </row>

</xml_diff>